<commit_message>
Reemplazar 'Cronograma de Actividades Completo.xlsx' con la versión corregida
</commit_message>
<xml_diff>
--- a/docs/Cronograma de Actividades Completo.xlsx
+++ b/docs/Cronograma de Actividades Completo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrie\OneDrive\Escritorio\Semestre 3\Programacion Orientada a Objetos\Proyecto tetris\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrie\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7AE6271-1763-4AF7-9C26-586832ABA605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BC3A0CC-A792-4BBC-A2D2-DA0DFE536148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{15099545-F71D-417F-811C-6FF15CA8FC0B}"/>
   </bookViews>
@@ -83,50 +83,20 @@
     <t>Versión final del juego Tetris Educativo lista para entrega y demostración.</t>
   </si>
   <si>
-    <t>• Agregar efectos sonoros y música de fondo.                       • Implementar opción de pausa y reanudación.                   • Pruebas integrales y corrección de errores.                         • Documentación final del proyecto.                                         • Presentación del producto terminado y retrospectiva Scrum.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">• Diseño y desarrollo de la pantalla de inicio (botón </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Jugar</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> y puntaje máximo).                                                                • Implementación de la cuadrícula central del juego.         • Programación del movimiento y rotación de piezas.       • Lógica para eliminar líneas completas.                                • Detección de Game Over al llenar una columna vertical.                                                                                                  • Pruebas de funcionamiento del juego base.</t>
-    </r>
-  </si>
-  <si>
     <t>• Implementación del sistema de niveles (10 niveles).      • Configuración de la dificultad progresiva (aumento de velocidad y operaciones más largas).                                      • Mostrar nivel actual y puntaje en pantalla (superior izquierda y derecha).                                                                        • Mostrar siguiente pieza en la parte inferior de la interfaz.                                                                                                  • Pruebas de estabilidad y jugabilidad.</t>
+  </si>
+  <si>
+    <t>• Diseño y desarrollo de la pantalla de inicio (botón Jugar e Instrucciones).                                                                    • Implementación de la cuadrícula central del juego.         • Programación del movimiento y rotación de piezas.       • Lógica para eliminar líneas completas.                                • Detección de Game Over al llenar una columna vertical.                                                                                                  • Pruebas de funcionamiento del juego base.</t>
+  </si>
+  <si>
+    <t>• Implementar opción de pausa y reanudación.                   • Pruebas integrales y corrección de errores.                         • Documentación final del proyecto.                                         • Presentación del producto terminado y retrospectiva Scrum.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,14 +106,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -176,10 +138,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -574,7 +536,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
@@ -594,7 +556,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -602,7 +564,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>14</v>

</xml_diff>